<commit_message>
Updating NBA data for March 28
</commit_message>
<xml_diff>
--- a/data/My_Hitter_Listing.xlsx
+++ b/data/My_Hitter_Listing.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29922"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29923"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Python\sports_dash_app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E34BC061-C39E-40D9-97A8-E58CF5525B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{38D3C13F-A836-4217-9A96-0041CA56665D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29765,7 +29765,7 @@
         <v>717</v>
       </c>
       <c r="B539" t="s">
-        <v>253</v>
+        <v>125</v>
       </c>
       <c r="C539" t="s">
         <v>254</v>
@@ -35992,7 +35992,7 @@
         <v>884</v>
       </c>
       <c r="B687" t="s">
-        <v>94</v>
+        <v>233</v>
       </c>
       <c r="C687" t="s">
         <v>95</v>
@@ -69760,7 +69760,7 @@
         <v>1781</v>
       </c>
       <c r="B1488" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="C1488" t="s">
         <v>68</v>
@@ -87632,7 +87632,7 @@
         <v>1557</v>
       </c>
       <c r="B1913" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C1913" t="s">
         <v>145</v>

</xml_diff>